<commit_message>
Officialbeurten: teamnamen normaliseren en nieuwe versie opgehaald
In de bron stonden "DS 9" en "Ds 9" naast elkaar; dat werden twee teams in de
filters en de telling klopte niet. Teamnamen worden nu genormaliseerd, waarmee
DS 9 op 14 beurten komt en het aantal teams van 38 naar 36 gaat.

Het live ophalen werkt weer: volevo.nl heeft het bestand opnieuw geplaatst
onder een andere naam (web2 in plaats van web), en doordat het script de link
van de pagina plukt kwam die nieuwe versie er vanzelf in. Verschil met de vorige:
twee telbeurten op 19 september van MB 3 naar JC 1 en JB 1 verplaatst.

Verder een controle die telt wanneer een team drie of meer officials tegelijk
moet leveren (19 keer). Ik had er eerst een waarschuwing van gemaakt vanaf twee
beurten, maar dat gebeurt 52 keer en is dus doodgewoon - dat zou alleen maar
ruis geven.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/officialbeurten.xlsx
+++ b/data/officialbeurten.xlsx
@@ -2,14 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
-  <fileSharing readOnlyRecommended="1"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Peter\Volevo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA7410A9-E8FD-4EC5-ABD1-51C9617C07EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5389F5C9-819F-4738-B7BB-C98DBCF1C711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -478,313 +477,313 @@
     <t>Kalinko MA 1</t>
   </si>
   <si>
+    <t>Zovoc MA 3</t>
+  </si>
+  <si>
+    <t>DS 6</t>
+  </si>
+  <si>
+    <t>VOLEVO MB 4</t>
+  </si>
+  <si>
+    <t>Zovoc MB 5</t>
+  </si>
+  <si>
+    <t>HS 6</t>
+  </si>
+  <si>
+    <t>VOLEVO MC 3</t>
+  </si>
+  <si>
+    <t>VVV Delta MC 1</t>
+  </si>
+  <si>
+    <t>JA 2</t>
+  </si>
+  <si>
+    <t>Zovoc MC 4</t>
+  </si>
+  <si>
+    <t>VOLEVO HS 1</t>
+  </si>
+  <si>
+    <t>Ancora RVV HS 1</t>
+  </si>
+  <si>
+    <t>dwf</t>
+  </si>
+  <si>
+    <t>JA 1</t>
+  </si>
+  <si>
+    <t>JB 2</t>
+  </si>
+  <si>
+    <t>VOLEVO JA 2</t>
+  </si>
+  <si>
+    <t>VCH JA 2</t>
+  </si>
+  <si>
+    <t>MC 3</t>
+  </si>
+  <si>
+    <t>Zovoc JB 2</t>
+  </si>
+  <si>
+    <t>Ancora RVV MC 1</t>
+  </si>
+  <si>
+    <t>MA 3</t>
+  </si>
+  <si>
+    <t>VOLEVO MA 5</t>
+  </si>
+  <si>
+    <t>WVV MA 1</t>
+  </si>
+  <si>
+    <t>HS 5</t>
+  </si>
+  <si>
+    <t>VOLEVO MC 2</t>
+  </si>
+  <si>
+    <t>Ancora RVV JC 1</t>
+  </si>
+  <si>
+    <t>VOLEVO DS 1</t>
+  </si>
+  <si>
+    <t>Van Rhijn Bouw Leython DC DS 2</t>
+  </si>
+  <si>
+    <t>VOLEVO HS 2</t>
+  </si>
+  <si>
+    <t>VELO HS 1</t>
+  </si>
+  <si>
+    <t>VOLEVO DS 5</t>
+  </si>
+  <si>
+    <t>SKC DS 6</t>
+  </si>
+  <si>
+    <t>scheidsrechter (vaardigheidstraining)</t>
+  </si>
+  <si>
+    <t>DS 7</t>
+  </si>
+  <si>
+    <t>VOLEVO DS 6</t>
+  </si>
+  <si>
+    <t>Kalinko DS 7</t>
+  </si>
+  <si>
+    <t>VOLEVO DS 8</t>
+  </si>
+  <si>
+    <t>Kratos '08 DS 6</t>
+  </si>
+  <si>
+    <t>VOLEVO HS 5</t>
+  </si>
+  <si>
+    <t>Punch HS 6</t>
+  </si>
+  <si>
+    <t>VOLEVO DS 7</t>
+  </si>
+  <si>
+    <t>VVV Delta DS 3</t>
+  </si>
+  <si>
+    <t>VOLEVO DS 9</t>
+  </si>
+  <si>
+    <t>Castellum DS 3</t>
+  </si>
+  <si>
+    <t>VOLEVO HS 4</t>
+  </si>
+  <si>
+    <t>Jupiter HS 2</t>
+  </si>
+  <si>
+    <t>Irene DS 1</t>
+  </si>
+  <si>
+    <t>VCS DS 1</t>
+  </si>
+  <si>
+    <t>VOLEVO HS 3</t>
+  </si>
+  <si>
+    <t>Volley2B HS 4</t>
+  </si>
+  <si>
+    <t>DEO HS 1</t>
+  </si>
+  <si>
+    <t>Zovoc MC 1</t>
+  </si>
+  <si>
+    <t>Kalinko MA 2</t>
+  </si>
+  <si>
+    <t>Ancora RVV MB 2</t>
+  </si>
+  <si>
+    <t>Sliedrecht Sport XC 1</t>
+  </si>
+  <si>
+    <t>ZVH MC 2</t>
+  </si>
+  <si>
+    <t>US DS 3</t>
+  </si>
+  <si>
+    <t>Next Volley Dordrecht HS 2</t>
+  </si>
+  <si>
+    <t>Dosko/Thor JA 1</t>
+  </si>
+  <si>
+    <t>MC 1</t>
+  </si>
+  <si>
+    <t>Leython DC MB 1</t>
+  </si>
+  <si>
+    <t>Netwerk JC 1</t>
+  </si>
+  <si>
+    <t>Zaanstad DS 3</t>
+  </si>
+  <si>
+    <t>Castellum JA 1</t>
+  </si>
+  <si>
+    <t>Netwerk MA 1</t>
+  </si>
+  <si>
+    <t>MA 4</t>
+  </si>
+  <si>
+    <t>Zovoc MB 3</t>
+  </si>
+  <si>
+    <t>Sovicos DS 3</t>
+  </si>
+  <si>
+    <t>Netwerk DS 1</t>
+  </si>
+  <si>
+    <t>Punch HS 5</t>
+  </si>
+  <si>
+    <t>VOLEVO HS 6</t>
+  </si>
+  <si>
+    <t>Monza HS 5</t>
+  </si>
+  <si>
+    <t>DEO DS 2</t>
+  </si>
+  <si>
+    <t>Inter Rijswijk DS 8</t>
+  </si>
+  <si>
+    <t>SKC HS 2</t>
+  </si>
+  <si>
+    <t>Sovicos DS 2</t>
+  </si>
+  <si>
+    <t>Sovicos DS 5</t>
+  </si>
+  <si>
+    <t>Sovicos DS 7</t>
+  </si>
+  <si>
+    <t>SKC HS 8</t>
+  </si>
+  <si>
+    <t>Limes MA 1</t>
+  </si>
+  <si>
+    <t>DEO MA 1</t>
+  </si>
+  <si>
+    <t>Kalinko MB 2</t>
+  </si>
+  <si>
+    <t>ZVH MB 2</t>
+  </si>
+  <si>
+    <t>Inter Rijswijk JC 1</t>
+  </si>
+  <si>
+    <t>Kratos '08 MC 1</t>
+  </si>
+  <si>
+    <t>Ancora RVV MC 3</t>
+  </si>
+  <si>
+    <t>Spaarnestad DS 3</t>
+  </si>
+  <si>
+    <t>MA 1</t>
+  </si>
+  <si>
+    <t>VHZ JB 1</t>
+  </si>
+  <si>
+    <t>Inter Rijswijk MA 2</t>
+  </si>
+  <si>
+    <t>Kratos '08 MA 1</t>
+  </si>
+  <si>
+    <t>Ancora RVV MB 1</t>
+  </si>
+  <si>
+    <t>Inter Rijswijk MB 2</t>
+  </si>
+  <si>
+    <t>ZVH JC 1</t>
+  </si>
+  <si>
+    <t>Inter Rijswijk JA 2</t>
+  </si>
+  <si>
+    <t>VELO JB 1</t>
+  </si>
+  <si>
+    <t>Inter Rijswijk MA 3</t>
+  </si>
+  <si>
+    <t>Zovoc DS 1</t>
+  </si>
+  <si>
+    <t>VollinGo HS 4</t>
+  </si>
+  <si>
+    <t>Zovoc DS 2</t>
+  </si>
+  <si>
+    <t>MC 2</t>
+  </si>
+  <si>
+    <t>Leython DC JA 2</t>
+  </si>
+  <si>
+    <t>Zovoc MA 2</t>
+  </si>
+  <si>
     <t>MB 3</t>
-  </si>
-  <si>
-    <t>Zovoc MA 3</t>
-  </si>
-  <si>
-    <t>DS 6</t>
-  </si>
-  <si>
-    <t>VOLEVO MB 4</t>
-  </si>
-  <si>
-    <t>Zovoc MB 5</t>
-  </si>
-  <si>
-    <t>HS 6</t>
-  </si>
-  <si>
-    <t>VOLEVO MC 3</t>
-  </si>
-  <si>
-    <t>VVV Delta MC 1</t>
-  </si>
-  <si>
-    <t>JA 2</t>
-  </si>
-  <si>
-    <t>Zovoc MC 4</t>
-  </si>
-  <si>
-    <t>VOLEVO HS 1</t>
-  </si>
-  <si>
-    <t>Ancora RVV HS 1</t>
-  </si>
-  <si>
-    <t>dwf</t>
-  </si>
-  <si>
-    <t>JA 1</t>
-  </si>
-  <si>
-    <t>JB 2</t>
-  </si>
-  <si>
-    <t>VOLEVO JA 2</t>
-  </si>
-  <si>
-    <t>VCH JA 2</t>
-  </si>
-  <si>
-    <t>MC 3</t>
-  </si>
-  <si>
-    <t>Zovoc JB 2</t>
-  </si>
-  <si>
-    <t>Ancora RVV MC 1</t>
-  </si>
-  <si>
-    <t>MA 3</t>
-  </si>
-  <si>
-    <t>VOLEVO MA 5</t>
-  </si>
-  <si>
-    <t>WVV MA 1</t>
-  </si>
-  <si>
-    <t>HS 5</t>
-  </si>
-  <si>
-    <t>VOLEVO MC 2</t>
-  </si>
-  <si>
-    <t>Ancora RVV JC 1</t>
-  </si>
-  <si>
-    <t>VOLEVO DS 1</t>
-  </si>
-  <si>
-    <t>Van Rhijn Bouw Leython DC DS 2</t>
-  </si>
-  <si>
-    <t>VOLEVO HS 2</t>
-  </si>
-  <si>
-    <t>VELO HS 1</t>
-  </si>
-  <si>
-    <t>VOLEVO DS 5</t>
-  </si>
-  <si>
-    <t>SKC DS 6</t>
-  </si>
-  <si>
-    <t>scheidsrechter (vaardigheidstraining)</t>
-  </si>
-  <si>
-    <t>DS 7</t>
-  </si>
-  <si>
-    <t>VOLEVO DS 6</t>
-  </si>
-  <si>
-    <t>Kalinko DS 7</t>
-  </si>
-  <si>
-    <t>VOLEVO DS 8</t>
-  </si>
-  <si>
-    <t>Kratos '08 DS 6</t>
-  </si>
-  <si>
-    <t>VOLEVO HS 5</t>
-  </si>
-  <si>
-    <t>Punch HS 6</t>
-  </si>
-  <si>
-    <t>VOLEVO DS 7</t>
-  </si>
-  <si>
-    <t>VVV Delta DS 3</t>
-  </si>
-  <si>
-    <t>VOLEVO DS 9</t>
-  </si>
-  <si>
-    <t>Castellum DS 3</t>
-  </si>
-  <si>
-    <t>VOLEVO HS 4</t>
-  </si>
-  <si>
-    <t>Jupiter HS 2</t>
-  </si>
-  <si>
-    <t>Irene DS 1</t>
-  </si>
-  <si>
-    <t>VCS DS 1</t>
-  </si>
-  <si>
-    <t>VOLEVO HS 3</t>
-  </si>
-  <si>
-    <t>Volley2B HS 4</t>
-  </si>
-  <si>
-    <t>DEO HS 1</t>
-  </si>
-  <si>
-    <t>Zovoc MC 1</t>
-  </si>
-  <si>
-    <t>Kalinko MA 2</t>
-  </si>
-  <si>
-    <t>Ancora RVV MB 2</t>
-  </si>
-  <si>
-    <t>Sliedrecht Sport XC 1</t>
-  </si>
-  <si>
-    <t>ZVH MC 2</t>
-  </si>
-  <si>
-    <t>US DS 3</t>
-  </si>
-  <si>
-    <t>Next Volley Dordrecht HS 2</t>
-  </si>
-  <si>
-    <t>Dosko/Thor JA 1</t>
-  </si>
-  <si>
-    <t>MC 1</t>
-  </si>
-  <si>
-    <t>Leython DC MB 1</t>
-  </si>
-  <si>
-    <t>Netwerk JC 1</t>
-  </si>
-  <si>
-    <t>Zaanstad DS 3</t>
-  </si>
-  <si>
-    <t>Castellum JA 1</t>
-  </si>
-  <si>
-    <t>Netwerk MA 1</t>
-  </si>
-  <si>
-    <t>MA 4</t>
-  </si>
-  <si>
-    <t>Zovoc MB 3</t>
-  </si>
-  <si>
-    <t>Sovicos DS 3</t>
-  </si>
-  <si>
-    <t>Netwerk DS 1</t>
-  </si>
-  <si>
-    <t>Punch HS 5</t>
-  </si>
-  <si>
-    <t>VOLEVO HS 6</t>
-  </si>
-  <si>
-    <t>Monza HS 5</t>
-  </si>
-  <si>
-    <t>DEO DS 2</t>
-  </si>
-  <si>
-    <t>Inter Rijswijk DS 8</t>
-  </si>
-  <si>
-    <t>SKC HS 2</t>
-  </si>
-  <si>
-    <t>Sovicos DS 2</t>
-  </si>
-  <si>
-    <t>Sovicos DS 5</t>
-  </si>
-  <si>
-    <t>Sovicos DS 7</t>
-  </si>
-  <si>
-    <t>SKC HS 8</t>
-  </si>
-  <si>
-    <t>Limes MA 1</t>
-  </si>
-  <si>
-    <t>DEO MA 1</t>
-  </si>
-  <si>
-    <t>Kalinko MB 2</t>
-  </si>
-  <si>
-    <t>ZVH MB 2</t>
-  </si>
-  <si>
-    <t>Inter Rijswijk JC 1</t>
-  </si>
-  <si>
-    <t>Kratos '08 MC 1</t>
-  </si>
-  <si>
-    <t>Ancora RVV MC 3</t>
-  </si>
-  <si>
-    <t>Spaarnestad DS 3</t>
-  </si>
-  <si>
-    <t>MA 1</t>
-  </si>
-  <si>
-    <t>VHZ JB 1</t>
-  </si>
-  <si>
-    <t>Inter Rijswijk MA 2</t>
-  </si>
-  <si>
-    <t>Kratos '08 MA 1</t>
-  </si>
-  <si>
-    <t>Ancora RVV MB 1</t>
-  </si>
-  <si>
-    <t>Inter Rijswijk MB 2</t>
-  </si>
-  <si>
-    <t>ZVH JC 1</t>
-  </si>
-  <si>
-    <t>Inter Rijswijk JA 2</t>
-  </si>
-  <si>
-    <t>VELO JB 1</t>
-  </si>
-  <si>
-    <t>Inter Rijswijk MA 3</t>
-  </si>
-  <si>
-    <t>Zovoc DS 1</t>
-  </si>
-  <si>
-    <t>VollinGo HS 4</t>
-  </si>
-  <si>
-    <t>Zovoc DS 2</t>
-  </si>
-  <si>
-    <t>MC 2</t>
-  </si>
-  <si>
-    <t>Leython DC JA 2</t>
-  </si>
-  <si>
-    <t>Zovoc MA 2</t>
   </si>
   <si>
     <t>Gemini-Kangeroes MB 1</t>
@@ -1025,7 +1024,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1107,6 +1106,13 @@
       <name val="Calibri"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1153,7 +1159,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1202,6 +1208,9 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -1627,7 +1636,7 @@
   <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.6328125" customWidth="1"/>
+    <col min="1" max="1" width="3.7265625" customWidth="1"/>
     <col min="2" max="2" width="132.453125" style="1" customWidth="1"/>
     <col min="3" max="3" width="3" customWidth="1"/>
   </cols>
@@ -1937,16 +1946,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16E71966-A700-42B0-97FD-F8A5129C645B}">
   <dimension ref="A1:J332"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.453125" style="13" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.453125" style="15" customWidth="1"/>
     <col min="3" max="3" width="17.54296875" style="15" customWidth="1"/>
-    <col min="4" max="4" width="36.36328125" style="15" customWidth="1"/>
-    <col min="5" max="5" width="34.36328125" style="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.26953125" style="15" customWidth="1"/>
+    <col min="5" max="5" width="34.26953125" style="15" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.453125" style="15" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="32.453125" style="15" customWidth="1"/>
-    <col min="8" max="16384" width="9.08984375" style="15"/>
+    <col min="8" max="16384" width="9.1796875" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -3044,8 +3053,8 @@
       <c r="E45" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="F45" s="15" t="s">
-        <v>104</v>
+      <c r="F45" s="20" t="s">
+        <v>85</v>
       </c>
       <c r="H45" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3063,13 +3072,13 @@
         <v>75</v>
       </c>
       <c r="D46" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="E46" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F46" s="15" t="s">
         <v>105</v>
-      </c>
-      <c r="E46" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F46" s="15" t="s">
-        <v>106</v>
       </c>
       <c r="H46" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3087,13 +3096,13 @@
         <v>75</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E47" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F47" s="15" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="H47" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3108,16 +3117,16 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C48" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D48" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="D48" s="15" t="s">
+      <c r="E48" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F48" s="15" t="s">
         <v>108</v>
-      </c>
-      <c r="E48" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F48" s="15" t="s">
-        <v>109</v>
       </c>
       <c r="H48" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3132,10 +3141,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C49" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D49" s="15" t="s">
         <v>107</v>
-      </c>
-      <c r="D49" s="15" t="s">
-        <v>108</v>
       </c>
       <c r="E49" s="15" t="s">
         <v>46</v>
@@ -3156,16 +3165,16 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C50" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="D50" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="D50" s="15" t="s">
+      <c r="E50" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F50" s="15" t="s">
         <v>111</v>
-      </c>
-      <c r="E50" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F50" s="15" t="s">
-        <v>112</v>
       </c>
       <c r="H50" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3180,10 +3189,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C51" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="D51" s="15" t="s">
         <v>110</v>
-      </c>
-      <c r="D51" s="15" t="s">
-        <v>111</v>
       </c>
       <c r="E51" s="15" t="s">
         <v>46</v>
@@ -3207,13 +3216,13 @@
         <v>96</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E52" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F52" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H52" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3231,7 +3240,7 @@
         <v>96</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E53" s="15" t="s">
         <v>46</v>
@@ -3252,16 +3261,16 @@
         <v>0.625</v>
       </c>
       <c r="C54" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="D54" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="D54" s="15" t="s">
+      <c r="E54" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="E54" s="15" t="s">
+      <c r="F54" s="15" t="s">
         <v>116</v>
-      </c>
-      <c r="F54" s="15" t="s">
-        <v>117</v>
       </c>
       <c r="H54" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3276,16 +3285,16 @@
         <v>0.625</v>
       </c>
       <c r="C55" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="D55" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="D55" s="15" t="s">
-        <v>115</v>
-      </c>
       <c r="E55" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F55" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H55" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3300,10 +3309,10 @@
         <v>0.625</v>
       </c>
       <c r="C56" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="D56" s="15" t="s">
         <v>119</v>
-      </c>
-      <c r="D56" s="15" t="s">
-        <v>120</v>
       </c>
       <c r="E56" s="15" t="s">
         <v>41</v>
@@ -3324,16 +3333,16 @@
         <v>0.625</v>
       </c>
       <c r="C57" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="D57" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="D57" s="15" t="s">
+      <c r="E57" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F57" s="15" t="s">
         <v>120</v>
-      </c>
-      <c r="E57" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F57" s="15" t="s">
-        <v>121</v>
       </c>
       <c r="H57" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3351,7 +3360,7 @@
         <v>48</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E58" s="15" t="s">
         <v>41</v>
@@ -3375,7 +3384,7 @@
         <v>48</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E59" s="15" t="s">
         <v>46</v>
@@ -3399,13 +3408,13 @@
         <v>65</v>
       </c>
       <c r="D60" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E60" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F60" s="15" t="s">
         <v>123</v>
-      </c>
-      <c r="E60" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F60" s="15" t="s">
-        <v>124</v>
       </c>
       <c r="H60" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3423,7 +3432,7 @@
         <v>65</v>
       </c>
       <c r="D61" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E61" s="15" t="s">
         <v>46</v>
@@ -3444,16 +3453,16 @@
         <v>0.625</v>
       </c>
       <c r="C62" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="D62" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="D62" s="15" t="s">
+      <c r="E62" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F62" s="15" t="s">
         <v>126</v>
-      </c>
-      <c r="E62" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F62" s="15" t="s">
-        <v>127</v>
       </c>
       <c r="H62" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3468,16 +3477,16 @@
         <v>0.625</v>
       </c>
       <c r="C63" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="D63" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="D63" s="15" t="s">
-        <v>126</v>
-      </c>
       <c r="E63" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F63" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H63" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3492,16 +3501,16 @@
         <v>0.625</v>
       </c>
       <c r="C64" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="D64" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="D64" s="15" t="s">
-        <v>129</v>
-      </c>
       <c r="E64" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F64" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H64" s="18" t="str">
         <f t="shared" si="0"/>
@@ -3516,10 +3525,10 @@
         <v>0.625</v>
       </c>
       <c r="C65" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="D65" s="15" t="s">
         <v>128</v>
-      </c>
-      <c r="D65" s="15" t="s">
-        <v>129</v>
       </c>
       <c r="E65" s="15" t="s">
         <v>46</v>
@@ -3540,13 +3549,13 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C66" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="D66" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="D66" s="15" t="s">
-        <v>131</v>
-      </c>
       <c r="E66" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F66" s="15" t="s">
         <v>45</v>
@@ -3564,10 +3573,10 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C67" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="D67" s="15" t="s">
         <v>130</v>
-      </c>
-      <c r="D67" s="15" t="s">
-        <v>131</v>
       </c>
       <c r="E67" s="15" t="s">
         <v>46</v>
@@ -3588,10 +3597,10 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C68" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="D68" s="15" t="s">
         <v>132</v>
-      </c>
-      <c r="D68" s="15" t="s">
-        <v>133</v>
       </c>
       <c r="E68" s="15" t="s">
         <v>46</v>
@@ -3612,13 +3621,13 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C69" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="D69" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="D69" s="15" t="s">
+      <c r="E69" s="15" t="s">
         <v>135</v>
-      </c>
-      <c r="E69" s="15" t="s">
-        <v>136</v>
       </c>
       <c r="F69" s="15" t="s">
         <v>77</v>
@@ -3636,16 +3645,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C70" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="D70" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="D70" s="15" t="s">
-        <v>135</v>
-      </c>
       <c r="E70" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F70" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H70" s="18" t="str">
         <f t="shared" si="1"/>
@@ -3660,13 +3669,13 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C71" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="D71" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="D71" s="15" t="s">
-        <v>139</v>
-      </c>
       <c r="E71" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F71" s="15" t="s">
         <v>77</v>
@@ -3684,16 +3693,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C72" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="D72" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="D72" s="15" t="s">
-        <v>139</v>
-      </c>
       <c r="E72" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F72" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H72" s="18" t="str">
         <f t="shared" si="1"/>
@@ -3708,16 +3717,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C73" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="D73" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="D73" s="15" t="s">
-        <v>141</v>
-      </c>
       <c r="E73" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F73" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H73" s="18" t="str">
         <f t="shared" si="1"/>
@@ -3732,10 +3741,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C74" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="D74" s="15" t="s">
         <v>140</v>
-      </c>
-      <c r="D74" s="15" t="s">
-        <v>141</v>
       </c>
       <c r="E74" s="15" t="s">
         <v>46</v>
@@ -3756,13 +3765,13 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C75" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="D75" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="D75" s="15" t="s">
-        <v>143</v>
-      </c>
       <c r="E75" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F75" s="15" t="s">
         <v>77</v>
@@ -3780,10 +3789,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C76" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="D76" s="15" t="s">
         <v>142</v>
-      </c>
-      <c r="D76" s="15" t="s">
-        <v>143</v>
       </c>
       <c r="E76" s="15" t="s">
         <v>46</v>
@@ -3804,13 +3813,13 @@
         <v>0.875</v>
       </c>
       <c r="C77" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="D77" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="D77" s="15" t="s">
-        <v>145</v>
-      </c>
       <c r="E77" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F77" s="15" t="s">
         <v>95</v>
@@ -3828,10 +3837,10 @@
         <v>0.875</v>
       </c>
       <c r="C78" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="D78" s="15" t="s">
         <v>144</v>
-      </c>
-      <c r="D78" s="15" t="s">
-        <v>145</v>
       </c>
       <c r="E78" s="15" t="s">
         <v>46</v>
@@ -3852,16 +3861,16 @@
         <v>0.875</v>
       </c>
       <c r="C79" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D79" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="D79" s="15" t="s">
-        <v>147</v>
-      </c>
       <c r="E79" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F79" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H79" s="18" t="str">
         <f t="shared" si="1"/>
@@ -3876,16 +3885,16 @@
         <v>0.875</v>
       </c>
       <c r="C80" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D80" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="D80" s="15" t="s">
-        <v>147</v>
-      </c>
       <c r="E80" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F80" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H80" s="18" t="str">
         <f t="shared" si="1"/>
@@ -3900,16 +3909,16 @@
         <v>0.875</v>
       </c>
       <c r="C81" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D81" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="D81" s="15" t="s">
-        <v>149</v>
-      </c>
       <c r="E81" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F81" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H81" s="18" t="str">
         <f t="shared" si="1"/>
@@ -3924,10 +3933,10 @@
         <v>0.875</v>
       </c>
       <c r="C82" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D82" s="15" t="s">
         <v>148</v>
-      </c>
-      <c r="D82" s="15" t="s">
-        <v>149</v>
       </c>
       <c r="E82" s="15" t="s">
         <v>46</v>
@@ -3951,7 +3960,7 @@
         <v>39</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E83" s="15" t="s">
         <v>46</v>
@@ -3975,7 +3984,7 @@
         <v>61</v>
       </c>
       <c r="D84" s="15" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E84" s="15" t="s">
         <v>46</v>
@@ -3996,13 +4005,13 @@
         <v>0.875</v>
       </c>
       <c r="C85" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D85" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="D85" s="15" t="s">
-        <v>153</v>
-      </c>
       <c r="E85" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F85" s="15" t="s">
         <v>45</v>
@@ -4020,10 +4029,10 @@
         <v>0.875</v>
       </c>
       <c r="C86" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D86" s="15" t="s">
         <v>152</v>
-      </c>
-      <c r="D86" s="15" t="s">
-        <v>153</v>
       </c>
       <c r="E86" s="15" t="s">
         <v>46</v>
@@ -4044,10 +4053,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C87" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E87" s="15" t="s">
         <v>46</v>
@@ -4071,13 +4080,13 @@
         <v>65</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E88" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F88" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H88" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4095,7 +4104,7 @@
         <v>65</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E89" s="15" t="s">
         <v>46</v>
@@ -4119,7 +4128,7 @@
         <v>52</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E90" s="15" t="s">
         <v>41</v>
@@ -4143,13 +4152,13 @@
         <v>52</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E91" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F91" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H91" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4167,7 +4176,7 @@
         <v>78</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E92" s="15" t="s">
         <v>41</v>
@@ -4191,7 +4200,7 @@
         <v>78</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E93" s="15" t="s">
         <v>46</v>
@@ -4215,7 +4224,7 @@
         <v>55</v>
       </c>
       <c r="D94" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E94" s="15" t="s">
         <v>41</v>
@@ -4242,7 +4251,7 @@
         <v>55</v>
       </c>
       <c r="D95" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E95" s="15" t="s">
         <v>46</v>
@@ -4266,13 +4275,13 @@
         <v>80</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E96" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F96" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H96" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4290,7 +4299,7 @@
         <v>80</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E97" s="15" t="s">
         <v>46</v>
@@ -4314,7 +4323,7 @@
         <v>58</v>
       </c>
       <c r="D98" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E98" s="15" t="s">
         <v>46</v>
@@ -4335,13 +4344,13 @@
         <v>0.625</v>
       </c>
       <c r="C99" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D99" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E99" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F99" s="15" t="s">
         <v>67</v>
@@ -4359,10 +4368,10 @@
         <v>0.625</v>
       </c>
       <c r="C100" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D100" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E100" s="15" t="s">
         <v>46</v>
@@ -4386,7 +4395,7 @@
         <v>43</v>
       </c>
       <c r="D101" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E101" s="15" t="s">
         <v>41</v>
@@ -4410,13 +4419,13 @@
         <v>43</v>
       </c>
       <c r="D102" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E102" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F102" s="15" t="s">
         <v>162</v>
-      </c>
-      <c r="E102" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F102" s="15" t="s">
-        <v>163</v>
       </c>
       <c r="H102" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4465,7 +4474,7 @@
         <v>46</v>
       </c>
       <c r="F104" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H104" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4483,7 +4492,7 @@
         <v>91</v>
       </c>
       <c r="D105" s="15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E105" s="15" t="s">
         <v>41</v>
@@ -4510,7 +4519,7 @@
         <v>91</v>
       </c>
       <c r="D106" s="15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E106" s="15" t="s">
         <v>46</v>
@@ -4531,10 +4540,10 @@
         <v>0.625</v>
       </c>
       <c r="C107" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D107" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E107" s="15" t="s">
         <v>41</v>
@@ -4555,10 +4564,10 @@
         <v>0.625</v>
       </c>
       <c r="C108" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D108" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E108" s="15" t="s">
         <v>46</v>
@@ -4579,16 +4588,16 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C109" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D109" s="15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E109" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F109" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H109" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4603,16 +4612,16 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C110" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D110" s="15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E110" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F110" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H110" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4627,10 +4636,10 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D111" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E111" s="15" t="s">
         <v>41</v>
@@ -4651,16 +4660,16 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C112" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D112" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E112" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F112" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H112" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4675,16 +4684,16 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C113" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D113" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E113" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F113" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H113" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4699,16 +4708,16 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C114" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D114" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E114" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F114" s="15" t="s">
         <v>168</v>
-      </c>
-      <c r="E114" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F114" s="15" t="s">
-        <v>169</v>
       </c>
       <c r="H114" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4726,7 +4735,7 @@
         <v>93</v>
       </c>
       <c r="D115" s="15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E115" s="15" t="s">
         <v>41</v>
@@ -4750,7 +4759,7 @@
         <v>93</v>
       </c>
       <c r="D116" s="15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E116" s="15" t="s">
         <v>46</v>
@@ -4771,16 +4780,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C117" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D117" s="15" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E117" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F117" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H117" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4795,16 +4804,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C118" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D118" s="15" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E118" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F118" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H118" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4819,10 +4828,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D119" s="15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E119" s="15" t="s">
         <v>41</v>
@@ -4843,10 +4852,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C120" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D120" s="15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E120" s="15" t="s">
         <v>46</v>
@@ -4867,16 +4876,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C121" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E121" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F121" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H121" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4891,16 +4900,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C122" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E122" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F122" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H122" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4915,16 +4924,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C123" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="D123" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="D123" s="15" t="s">
-        <v>175</v>
-      </c>
       <c r="E123" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F123" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H123" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4939,16 +4948,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C124" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="D124" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="D124" s="15" t="s">
-        <v>175</v>
-      </c>
       <c r="E124" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F124" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H124" s="18" t="str">
         <f t="shared" si="1"/>
@@ -4963,13 +4972,13 @@
         <v>0.875</v>
       </c>
       <c r="C125" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D125" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E125" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F125" s="15" t="s">
         <v>77</v>
@@ -4987,10 +4996,10 @@
         <v>0.875</v>
       </c>
       <c r="C126" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D126" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E126" s="15" t="s">
         <v>46</v>
@@ -5011,16 +5020,16 @@
         <v>0.875</v>
       </c>
       <c r="C127" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D127" s="15" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E127" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F127" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H127" s="18" t="str">
         <f t="shared" si="1"/>
@@ -5035,16 +5044,16 @@
         <v>0.875</v>
       </c>
       <c r="C128" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D128" s="15" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E128" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F128" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H128" s="18" t="str">
         <f t="shared" si="1"/>
@@ -5059,13 +5068,13 @@
         <v>0.875</v>
       </c>
       <c r="C129" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D129" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E129" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F129" s="15" t="s">
         <v>77</v>
@@ -5083,16 +5092,16 @@
         <v>0.875</v>
       </c>
       <c r="C130" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D130" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E130" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F130" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H130" s="18" t="str">
         <f t="shared" si="1"/>
@@ -5107,13 +5116,13 @@
         <v>0.875</v>
       </c>
       <c r="C131" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D131" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E131" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F131" s="15" t="s">
         <v>45</v>
@@ -5131,10 +5140,10 @@
         <v>0.875</v>
       </c>
       <c r="C132" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D132" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E132" s="15" t="s">
         <v>46</v>
@@ -5155,13 +5164,13 @@
         <v>0.875</v>
       </c>
       <c r="C133" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D133" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E133" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F133" s="15" t="s">
         <v>88</v>
@@ -5179,10 +5188,10 @@
         <v>0.875</v>
       </c>
       <c r="C134" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D134" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E134" s="15" t="s">
         <v>46</v>
@@ -5203,16 +5212,16 @@
         <v>0.875</v>
       </c>
       <c r="C135" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D135" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E135" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F135" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H135" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5227,16 +5236,16 @@
         <v>0.875</v>
       </c>
       <c r="C136" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D136" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E136" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F136" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H136" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5251,10 +5260,10 @@
         <v>0.875</v>
       </c>
       <c r="C137" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D137" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E137" s="15" t="s">
         <v>41</v>
@@ -5275,16 +5284,16 @@
         <v>0.875</v>
       </c>
       <c r="C138" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D138" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E138" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F138" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H138" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5302,7 +5311,7 @@
         <v>68</v>
       </c>
       <c r="D139" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E139" s="15" t="s">
         <v>41</v>
@@ -5329,7 +5338,7 @@
         <v>68</v>
       </c>
       <c r="D140" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E140" s="15" t="s">
         <v>46</v>
@@ -5350,16 +5359,16 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C141" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D141" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E141" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F141" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H141" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5374,10 +5383,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C142" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D142" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E142" s="15" t="s">
         <v>46</v>
@@ -5401,7 +5410,7 @@
         <v>78</v>
       </c>
       <c r="D143" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E143" s="15" t="s">
         <v>41</v>
@@ -5425,7 +5434,7 @@
         <v>78</v>
       </c>
       <c r="D144" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E144" s="15" t="s">
         <v>46</v>
@@ -5446,16 +5455,16 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C145" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D145" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E145" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F145" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H145" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5470,10 +5479,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C146" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D146" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E146" s="15" t="s">
         <v>46</v>
@@ -5497,7 +5506,7 @@
         <v>55</v>
       </c>
       <c r="D147" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E147" s="15" t="s">
         <v>41</v>
@@ -5524,7 +5533,7 @@
         <v>55</v>
       </c>
       <c r="D148" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E148" s="15" t="s">
         <v>46</v>
@@ -5545,16 +5554,16 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C149" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D149" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E149" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F149" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H149" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5569,10 +5578,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C150" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D150" s="15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E150" s="15" t="s">
         <v>46</v>
@@ -5596,13 +5605,13 @@
         <v>96</v>
       </c>
       <c r="D151" s="15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E151" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F151" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H151" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5620,7 +5629,7 @@
         <v>96</v>
       </c>
       <c r="D152" s="15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E152" s="15" t="s">
         <v>46</v>
@@ -5644,13 +5653,13 @@
         <v>58</v>
       </c>
       <c r="D153" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="E153" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F153" s="15" t="s">
         <v>190</v>
-      </c>
-      <c r="E153" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F153" s="15" t="s">
-        <v>191</v>
       </c>
       <c r="H153" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5668,7 +5677,7 @@
         <v>48</v>
       </c>
       <c r="D154" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E154" s="15" t="s">
         <v>41</v>
@@ -5692,7 +5701,7 @@
         <v>48</v>
       </c>
       <c r="D155" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E155" s="15" t="s">
         <v>46</v>
@@ -5716,7 +5725,7 @@
         <v>71</v>
       </c>
       <c r="D156" s="15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E156" s="15" t="s">
         <v>41</v>
@@ -5740,13 +5749,13 @@
         <v>71</v>
       </c>
       <c r="D157" s="15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E157" s="15" t="s">
         <v>46</v>
       </c>
       <c r="F157" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H157" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5764,13 +5773,13 @@
         <v>75</v>
       </c>
       <c r="D158" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E158" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F158" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H158" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5788,7 +5797,7 @@
         <v>75</v>
       </c>
       <c r="D159" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E159" s="15" t="s">
         <v>46</v>
@@ -5812,7 +5821,7 @@
         <v>91</v>
       </c>
       <c r="D160" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E160" s="15" t="s">
         <v>41</v>
@@ -5839,7 +5848,7 @@
         <v>91</v>
       </c>
       <c r="D161" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E161" s="15" t="s">
         <v>46</v>
@@ -5863,7 +5872,7 @@
         <v>93</v>
       </c>
       <c r="D162" s="15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E162" s="15" t="s">
         <v>41</v>
@@ -5887,7 +5896,7 @@
         <v>93</v>
       </c>
       <c r="D163" s="15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E163" s="15" t="s">
         <v>46</v>
@@ -5908,16 +5917,16 @@
         <v>0.625</v>
       </c>
       <c r="C164" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D164" s="15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E164" s="15" t="s">
         <v>41</v>
       </c>
       <c r="F164" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H164" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5932,10 +5941,10 @@
         <v>0.625</v>
       </c>
       <c r="C165" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D165" s="15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E165" s="15" t="s">
         <v>46</v>
@@ -5959,7 +5968,7 @@
         <v>43</v>
       </c>
       <c r="D166" s="15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E166" s="15" t="s">
         <v>41</v>
@@ -5983,7 +5992,7 @@
         <v>43</v>
       </c>
       <c r="D167" s="15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E167" s="15" t="s">
         <v>46</v>
@@ -6007,7 +6016,7 @@
         <v>86</v>
       </c>
       <c r="D168" s="15" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E168" s="15" t="s">
         <v>41</v>
@@ -6031,7 +6040,7 @@
         <v>86</v>
       </c>
       <c r="D169" s="15" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E169" s="15" t="s">
         <v>46</v>
@@ -6055,7 +6064,7 @@
         <v>52</v>
       </c>
       <c r="D170" s="15" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E170" s="15" t="s">
         <v>41</v>
@@ -6079,7 +6088,7 @@
         <v>52</v>
       </c>
       <c r="D171" s="15" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E171" s="15" t="s">
         <v>46</v>
@@ -6103,7 +6112,7 @@
         <v>39</v>
       </c>
       <c r="D172" s="15" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E172" s="15" t="s">
         <v>46</v>
@@ -6124,13 +6133,13 @@
         <v>0.875</v>
       </c>
       <c r="C173" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D173" s="15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E173" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F173" s="15" t="s">
         <v>45</v>
@@ -6148,10 +6157,10 @@
         <v>0.875</v>
       </c>
       <c r="C174" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D174" s="15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E174" s="15" t="s">
         <v>46</v>
@@ -6175,13 +6184,13 @@
         <v>61</v>
       </c>
       <c r="D175" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="E175" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F175" s="15" t="s">
         <v>203</v>
-      </c>
-      <c r="E175" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F175" s="15" t="s">
-        <v>204</v>
       </c>
       <c r="H175" s="18" t="str">
         <f t="shared" si="2"/>
@@ -6196,10 +6205,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C176" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D176" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E176" s="15" t="s">
         <v>41</v>
@@ -6220,10 +6229,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C177" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D177" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E177" s="15" t="s">
         <v>46</v>
@@ -6247,7 +6256,7 @@
         <v>52</v>
       </c>
       <c r="D178" s="15" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E178" s="15" t="s">
         <v>41</v>
@@ -6271,13 +6280,13 @@
         <v>52</v>
       </c>
       <c r="D179" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="E179" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F179" s="15" t="s">
         <v>206</v>
-      </c>
-      <c r="E179" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F179" s="15" t="s">
-        <v>104</v>
       </c>
       <c r="H179" s="18" t="str">
         <f t="shared" si="2"/>
@@ -6340,7 +6349,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C182" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D182" s="15" t="s">
         <v>208</v>
@@ -6364,7 +6373,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C183" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D183" s="15" t="s">
         <v>208</v>
@@ -6448,7 +6457,7 @@
         <v>41</v>
       </c>
       <c r="F186" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H186" s="18" t="str">
         <f t="shared" si="2"/>
@@ -6487,13 +6496,13 @@
         <v>0.625</v>
       </c>
       <c r="C188" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D188" s="15" t="s">
         <v>211</v>
       </c>
       <c r="E188" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F188" s="15" t="s">
         <v>50</v>
@@ -6511,7 +6520,7 @@
         <v>0.625</v>
       </c>
       <c r="C189" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D189" s="15" t="s">
         <v>211</v>
@@ -6538,7 +6547,7 @@
         <v>102</v>
       </c>
       <c r="D190" s="15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E190" s="15" t="s">
         <v>41</v>
@@ -6562,7 +6571,7 @@
         <v>102</v>
       </c>
       <c r="D191" s="15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E191" s="15" t="s">
         <v>46</v>
@@ -6730,7 +6739,7 @@
         <v>0.625</v>
       </c>
       <c r="C198" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D198" s="15" t="s">
         <v>56</v>
@@ -6739,7 +6748,7 @@
         <v>41</v>
       </c>
       <c r="F198" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H198" s="18" t="str">
         <f t="shared" si="3"/>
@@ -6754,7 +6763,7 @@
         <v>0.625</v>
       </c>
       <c r="C199" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D199" s="15" t="s">
         <v>56</v>
@@ -6778,13 +6787,13 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C200" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D200" s="15" t="s">
         <v>217</v>
       </c>
       <c r="E200" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F200" s="15" t="s">
         <v>45</v>
@@ -6802,7 +6811,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C201" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D201" s="15" t="s">
         <v>217</v>
@@ -6811,7 +6820,7 @@
         <v>46</v>
       </c>
       <c r="F201" s="15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H201" s="18" t="str">
         <f t="shared" si="3"/>
@@ -6826,7 +6835,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C202" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D202" s="15" t="s">
         <v>218</v>
@@ -6874,13 +6883,13 @@
         <v>0.875</v>
       </c>
       <c r="C204" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D204" s="15" t="s">
         <v>220</v>
       </c>
       <c r="E204" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F204" s="15" t="s">
         <v>45</v>
@@ -6898,7 +6907,7 @@
         <v>0.875</v>
       </c>
       <c r="C205" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D205" s="15" t="s">
         <v>220</v>
@@ -6931,7 +6940,7 @@
         <v>46</v>
       </c>
       <c r="F206" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H206" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7042,7 +7051,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C211" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D211" s="15" t="s">
         <v>223</v>
@@ -7051,7 +7060,7 @@
         <v>41</v>
       </c>
       <c r="F211" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H211" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7066,7 +7075,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C212" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D212" s="15" t="s">
         <v>223</v>
@@ -7075,7 +7084,7 @@
         <v>46</v>
       </c>
       <c r="F212" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H212" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7141,7 +7150,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C215" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D215" s="15" t="s">
         <v>225</v>
@@ -7150,7 +7159,7 @@
         <v>41</v>
       </c>
       <c r="F215" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H215" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7165,7 +7174,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C216" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D216" s="15" t="s">
         <v>225</v>
@@ -7189,7 +7198,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C217" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D217" s="15" t="s">
         <v>226</v>
@@ -7198,7 +7207,7 @@
         <v>41</v>
       </c>
       <c r="F217" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H217" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7213,7 +7222,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C218" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D218" s="15" t="s">
         <v>226</v>
@@ -7237,13 +7246,13 @@
         <v>0.625</v>
       </c>
       <c r="C219" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="D219" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="D219" s="15" t="s">
+      <c r="E219" s="15" t="s">
         <v>115</v>
-      </c>
-      <c r="E219" s="15" t="s">
-        <v>116</v>
       </c>
       <c r="F219" s="15" t="s">
         <v>50</v>
@@ -7261,10 +7270,10 @@
         <v>0.625</v>
       </c>
       <c r="C220" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="D220" s="15" t="s">
         <v>114</v>
-      </c>
-      <c r="D220" s="15" t="s">
-        <v>115</v>
       </c>
       <c r="E220" s="15" t="s">
         <v>46</v>
@@ -7366,7 +7375,7 @@
         <v>46</v>
       </c>
       <c r="F224" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H224" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7390,7 +7399,7 @@
         <v>41</v>
       </c>
       <c r="F225" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H225" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7438,7 +7447,7 @@
         <v>41</v>
       </c>
       <c r="F227" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H227" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7477,13 +7486,13 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C229" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D229" s="15" t="s">
         <v>230</v>
       </c>
       <c r="E229" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F229" s="15" t="s">
         <v>67</v>
@@ -7501,7 +7510,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C230" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D230" s="15" t="s">
         <v>230</v>
@@ -7525,7 +7534,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C231" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D231" s="15" t="s">
         <v>232</v>
@@ -7534,7 +7543,7 @@
         <v>46</v>
       </c>
       <c r="F231" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H231" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7549,13 +7558,13 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C232" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D232" s="15" t="s">
         <v>233</v>
       </c>
       <c r="E232" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F232" s="15" t="s">
         <v>88</v>
@@ -7573,7 +7582,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C233" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D233" s="15" t="s">
         <v>233</v>
@@ -7597,13 +7606,13 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C234" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D234" s="15" t="s">
         <v>234</v>
       </c>
       <c r="E234" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F234" s="15" t="s">
         <v>88</v>
@@ -7621,7 +7630,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C235" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D235" s="15" t="s">
         <v>234</v>
@@ -7696,7 +7705,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C238" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D238" s="15" t="s">
         <v>236</v>
@@ -7705,7 +7714,7 @@
         <v>41</v>
       </c>
       <c r="F238" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H238" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7720,7 +7729,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C239" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D239" s="15" t="s">
         <v>236</v>
@@ -7753,7 +7762,7 @@
         <v>46</v>
       </c>
       <c r="F240" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H240" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7768,13 +7777,13 @@
         <v>0.875</v>
       </c>
       <c r="C241" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D241" s="15" t="s">
         <v>238</v>
       </c>
       <c r="E241" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F241" s="15" t="s">
         <v>77</v>
@@ -7792,7 +7801,7 @@
         <v>0.875</v>
       </c>
       <c r="C242" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D242" s="15" t="s">
         <v>238</v>
@@ -7801,7 +7810,7 @@
         <v>46</v>
       </c>
       <c r="F242" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H242" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7816,7 +7825,7 @@
         <v>0.875</v>
       </c>
       <c r="C243" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D243" s="15" t="s">
         <v>239</v>
@@ -7840,7 +7849,7 @@
         <v>0.875</v>
       </c>
       <c r="C244" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D244" s="15" t="s">
         <v>239</v>
@@ -7864,13 +7873,13 @@
         <v>0.875</v>
       </c>
       <c r="C245" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D245" s="15" t="s">
         <v>240</v>
       </c>
       <c r="E245" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F245" s="15" t="s">
         <v>77</v>
@@ -7888,7 +7897,7 @@
         <v>0.875</v>
       </c>
       <c r="C246" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D246" s="15" t="s">
         <v>240</v>
@@ -7897,7 +7906,7 @@
         <v>46</v>
       </c>
       <c r="F246" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H246" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7912,7 +7921,7 @@
         <v>0.875</v>
       </c>
       <c r="C247" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D247" s="15" t="s">
         <v>241</v>
@@ -7936,7 +7945,7 @@
         <v>0.875</v>
       </c>
       <c r="C248" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D248" s="15" t="s">
         <v>241</v>
@@ -7984,13 +7993,13 @@
         <v>0.875</v>
       </c>
       <c r="C250" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D250" s="15" t="s">
         <v>243</v>
       </c>
       <c r="E250" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F250" s="15" t="s">
         <v>45</v>
@@ -8008,7 +8017,7 @@
         <v>0.875</v>
       </c>
       <c r="C251" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D251" s="15" t="s">
         <v>243</v>
@@ -8032,7 +8041,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C252" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D252" s="15" t="s">
         <v>244</v>
@@ -8113,7 +8122,7 @@
         <v>41</v>
       </c>
       <c r="F255" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H255" s="18" t="str">
         <f t="shared" si="3"/>
@@ -8185,7 +8194,7 @@
         <v>46</v>
       </c>
       <c r="F258" s="15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H258" s="18" t="str">
         <f t="shared" si="3"/>
@@ -8260,7 +8269,7 @@
         <v>41</v>
       </c>
       <c r="F261" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H261" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8347,16 +8356,16 @@
         <v>0.625</v>
       </c>
       <c r="C265" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D265" s="15" t="s">
         <v>250</v>
       </c>
       <c r="E265" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="F265" s="15" t="s">
         <v>116</v>
-      </c>
-      <c r="F265" s="15" t="s">
-        <v>117</v>
       </c>
       <c r="H265" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8371,7 +8380,7 @@
         <v>0.625</v>
       </c>
       <c r="C266" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D266" s="15" t="s">
         <v>250</v>
@@ -8395,7 +8404,7 @@
         <v>0.625</v>
       </c>
       <c r="C267" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D267" s="15" t="s">
         <v>251</v>
@@ -8419,7 +8428,7 @@
         <v>0.625</v>
       </c>
       <c r="C268" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D268" s="15" t="s">
         <v>251</v>
@@ -8428,7 +8437,7 @@
         <v>46</v>
       </c>
       <c r="F268" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H268" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8443,7 +8452,7 @@
         <v>0.625</v>
       </c>
       <c r="C269" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D269" s="15" t="s">
         <v>252</v>
@@ -8452,7 +8461,7 @@
         <v>41</v>
       </c>
       <c r="F269" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H269" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8467,7 +8476,7 @@
         <v>0.625</v>
       </c>
       <c r="C270" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D270" s="15" t="s">
         <v>252</v>
@@ -8500,7 +8509,7 @@
         <v>41</v>
       </c>
       <c r="F271" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H271" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8539,16 +8548,16 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C273" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D273" s="15" t="s">
         <v>254</v>
       </c>
       <c r="E273" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F273" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H273" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8563,7 +8572,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C274" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D274" s="15" t="s">
         <v>254</v>
@@ -8572,7 +8581,7 @@
         <v>46</v>
       </c>
       <c r="F274" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H274" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8620,7 +8629,7 @@
         <v>46</v>
       </c>
       <c r="F276" s="15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H276" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8644,7 +8653,7 @@
         <v>41</v>
       </c>
       <c r="F277" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H277" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8692,7 +8701,7 @@
         <v>41</v>
       </c>
       <c r="F279" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H279" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8731,7 +8740,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C281" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D281" s="15" t="s">
         <v>258</v>
@@ -8740,7 +8749,7 @@
         <v>41</v>
       </c>
       <c r="F281" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H281" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8755,7 +8764,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C282" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D282" s="15" t="s">
         <v>258</v>
@@ -8779,16 +8788,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C283" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D283" s="15" t="s">
         <v>259</v>
       </c>
       <c r="E283" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F283" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H283" s="18" t="str">
         <f t="shared" si="4"/>
@@ -8803,7 +8812,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C284" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D284" s="15" t="s">
         <v>259</v>
@@ -8827,7 +8836,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C285" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D285" s="15" t="s">
         <v>261</v>
@@ -8851,7 +8860,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="C286" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D286" s="15" t="s">
         <v>261</v>
@@ -8935,7 +8944,7 @@
         <v>41</v>
       </c>
       <c r="F289" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G289" s="15" t="s">
         <v>57</v>
@@ -8977,13 +8986,13 @@
         <v>0.875</v>
       </c>
       <c r="C291" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D291" s="15" t="s">
         <v>264</v>
       </c>
       <c r="E291" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F291" s="15" t="s">
         <v>88</v>
@@ -9001,7 +9010,7 @@
         <v>0.875</v>
       </c>
       <c r="C292" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D292" s="15" t="s">
         <v>264</v>
@@ -9010,7 +9019,7 @@
         <v>46</v>
       </c>
       <c r="F292" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H292" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9025,16 +9034,16 @@
         <v>0.875</v>
       </c>
       <c r="C293" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D293" s="15" t="s">
         <v>265</v>
       </c>
       <c r="E293" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="F293" s="15" t="s">
         <v>136</v>
-      </c>
-      <c r="F293" s="15" t="s">
-        <v>137</v>
       </c>
       <c r="H293" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9049,7 +9058,7 @@
         <v>0.875</v>
       </c>
       <c r="C294" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D294" s="15" t="s">
         <v>265</v>
@@ -9058,7 +9067,7 @@
         <v>46</v>
       </c>
       <c r="F294" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H294" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9073,7 +9082,7 @@
         <v>0.875</v>
       </c>
       <c r="C295" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D295" s="15" t="s">
         <v>266</v>
@@ -9097,7 +9106,7 @@
         <v>0.875</v>
       </c>
       <c r="C296" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D296" s="15" t="s">
         <v>266</v>
@@ -9121,13 +9130,13 @@
         <v>0.875</v>
       </c>
       <c r="C297" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D297" s="15" t="s">
         <v>267</v>
       </c>
       <c r="E297" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F297" s="15" t="s">
         <v>45</v>
@@ -9145,7 +9154,7 @@
         <v>0.875</v>
       </c>
       <c r="C298" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D298" s="15" t="s">
         <v>267</v>
@@ -9178,7 +9187,7 @@
         <v>41</v>
       </c>
       <c r="F299" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H299" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9226,7 +9235,7 @@
         <v>46</v>
       </c>
       <c r="F301" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H301" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9265,13 +9274,13 @@
         <v>0.875</v>
       </c>
       <c r="C303" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D303" s="15" t="s">
         <v>271</v>
       </c>
       <c r="E303" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F303" s="15" t="s">
         <v>45</v>
@@ -9289,7 +9298,7 @@
         <v>0.875</v>
       </c>
       <c r="C304" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D304" s="15" t="s">
         <v>271</v>
@@ -9337,7 +9346,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C306" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D306" s="15" t="s">
         <v>273</v>
@@ -9361,7 +9370,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C307" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D307" s="15" t="s">
         <v>273</v>
@@ -9484,7 +9493,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C312" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D312" s="15" t="s">
         <v>275</v>
@@ -9493,7 +9502,7 @@
         <v>41</v>
       </c>
       <c r="F312" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H312" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9508,7 +9517,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C313" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D313" s="15" t="s">
         <v>275</v>
@@ -9517,7 +9526,7 @@
         <v>46</v>
       </c>
       <c r="F313" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H313" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9541,7 +9550,7 @@
         <v>41</v>
       </c>
       <c r="F314" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H314" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9580,7 +9589,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C316" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D316" s="15" t="s">
         <v>277</v>
@@ -9589,7 +9598,7 @@
         <v>41</v>
       </c>
       <c r="F316" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H316" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9604,7 +9613,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="C317" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D317" s="15" t="s">
         <v>277</v>
@@ -9628,16 +9637,16 @@
         <v>0.625</v>
       </c>
       <c r="C318" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D318" s="15" t="s">
         <v>278</v>
       </c>
       <c r="E318" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F318" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H318" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9652,7 +9661,7 @@
         <v>0.625</v>
       </c>
       <c r="C319" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D319" s="15" t="s">
         <v>278</v>
@@ -9661,7 +9670,7 @@
         <v>46</v>
       </c>
       <c r="F319" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H319" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9709,7 +9718,7 @@
         <v>46</v>
       </c>
       <c r="F321" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H321" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9733,7 +9742,7 @@
         <v>41</v>
       </c>
       <c r="F322" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H322" s="18" t="str">
         <f t="shared" si="4"/>
@@ -9772,16 +9781,16 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C324" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D324" s="15" t="s">
         <v>280</v>
       </c>
       <c r="E324" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F324" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H324" s="18" t="str">
         <f t="shared" si="5"/>
@@ -9796,7 +9805,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C325" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D325" s="15" t="s">
         <v>280</v>
@@ -9805,7 +9814,7 @@
         <v>46</v>
       </c>
       <c r="F325" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H325" s="18" t="str">
         <f t="shared" si="5"/>
@@ -9820,7 +9829,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="C326" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D326" s="15" t="s">
         <v>281</v>
@@ -9829,7 +9838,7 @@
         <v>46</v>
       </c>
       <c r="F326" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H326" s="18" t="str">
         <f t="shared" si="5"/>
@@ -9844,13 +9853,13 @@
         <v>0.875</v>
       </c>
       <c r="C327" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D327" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E327" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F327" s="15" t="s">
         <v>73</v>
@@ -9868,10 +9877,10 @@
         <v>0.875</v>
       </c>
       <c r="C328" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D328" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E328" s="15" t="s">
         <v>46</v>
@@ -9892,13 +9901,13 @@
         <v>0.875</v>
       </c>
       <c r="C329" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D329" s="15" t="s">
         <v>282</v>
       </c>
       <c r="E329" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F329" s="15" t="s">
         <v>90</v>
@@ -9916,7 +9925,7 @@
         <v>0.875</v>
       </c>
       <c r="C330" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D330" s="15" t="s">
         <v>282</v>
@@ -9940,7 +9949,7 @@
         <v>0.875</v>
       </c>
       <c r="C331" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D331" s="15" t="s">
         <v>283</v>
@@ -9949,7 +9958,7 @@
         <v>41</v>
       </c>
       <c r="F331" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H331" s="18" t="str">
         <f t="shared" si="5"/>
@@ -9964,7 +9973,7 @@
         <v>0.875</v>
       </c>
       <c r="C332" s="15" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D332" s="15" t="s">
         <v>283</v>
@@ -9973,7 +9982,7 @@
         <v>46</v>
       </c>
       <c r="F332" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H332" s="18" t="str">
         <f t="shared" si="5"/>

</xml_diff>